<commit_message>
Updated data files because for some reason we track them.
</commit_message>
<xml_diff>
--- a/corr_matrix/residual_exam1A_1PL.xlsx
+++ b/corr_matrix/residual_exam1A_1PL.xlsx
@@ -429,6 +429,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>question_id</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>1A01</t>
@@ -520,49 +525,49 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.1714310713673903</v>
+        <v>-0.1714354285074073</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.03989991096810733</v>
+        <v>-0.03990355705902224</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1122395588124433</v>
+        <v>-0.1122229579496982</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.09616081275407345</v>
+        <v>-0.09614653193185965</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.1096170365425155</v>
+        <v>-0.1096135312118162</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.1444223790502424</v>
+        <v>-0.1444150351135369</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.1096209680711279</v>
+        <v>-0.1096233308647602</v>
       </c>
       <c r="J2" t="n">
-        <v>0.04925957383564745</v>
+        <v>0.04925397476812462</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03502995936437731</v>
+        <v>0.03502673390221027</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.07146579894713018</v>
+        <v>-0.07146496179968009</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.1641235860623537</v>
+        <v>-0.1641089118636049</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.1415073162202437</v>
+        <v>-0.1415288649930178</v>
       </c>
       <c r="O2" t="n">
-        <v>0.08680963195490667</v>
+        <v>0.08680258700840175</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.09777156231626215</v>
+        <v>-0.09775477875327418</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.04353341731158855</v>
+        <v>0.04354939586290017</v>
       </c>
     </row>
     <row r="3">
@@ -572,52 +577,52 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.1714310713673903</v>
+        <v>-0.1714354285074073</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.01828652680198198</v>
+        <v>-0.01829149861193519</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1024485772601533</v>
+        <v>-0.1024488456682838</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.08689012223718132</v>
+        <v>-0.08689302559642334</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.02214946444162377</v>
+        <v>-0.02216192929112734</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1667356404338387</v>
+        <v>0.1667294725423881</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.1285428703752398</v>
+        <v>-0.1285498004740148</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.04364093524481442</v>
+        <v>-0.04363539419800175</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.01414280009000239</v>
+        <v>-0.01414764888703375</v>
       </c>
       <c r="L3" t="n">
-        <v>0.08837535754800829</v>
+        <v>0.08833101272917128</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.0003000413873512097</v>
+        <v>-0.0003130020767969113</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.01353837558253563</v>
+        <v>-0.01354378942813579</v>
       </c>
       <c r="O3" t="n">
-        <v>-0.1815010411147558</v>
+        <v>-0.1815036698852637</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.2443966077704177</v>
+        <v>-0.2443978567840111</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.2406847034745391</v>
+        <v>-0.2406974875923396</v>
       </c>
     </row>
     <row r="4">
@@ -627,52 +632,52 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.03989991096810733</v>
+        <v>-0.03990355705902224</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.01828652680198198</v>
+        <v>-0.01829149861193519</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01863422289755997</v>
+        <v>0.01862259318770651</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1024578075750018</v>
+        <v>-0.1024670641381996</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.09036043017487924</v>
+        <v>-0.09035629639522169</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.259347697756791</v>
+        <v>-0.2593522376531645</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.06117100019707069</v>
+        <v>-0.06118335721699146</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1082913665113159</v>
+        <v>0.1082970332787706</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.05702846365874022</v>
+        <v>-0.05702766288127244</v>
       </c>
       <c r="L4" t="n">
-        <v>0.07834398564172869</v>
+        <v>0.07834318818553589</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.138863151511475</v>
+        <v>-0.1388742670750134</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.1644678256392396</v>
+        <v>-0.1644710669846303</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0207348601794416</v>
+        <v>0.02073547525390141</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.0128512565357735</v>
+        <v>-0.01285610416450294</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.134669307620711</v>
+        <v>-0.1346716575196713</v>
       </c>
     </row>
     <row r="5">
@@ -682,52 +687,52 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.1122395588124433</v>
+        <v>-0.1122229579496982</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.1024485772601533</v>
+        <v>-0.1024488456682838</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01863422289755997</v>
+        <v>0.01862259318770651</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.2398266474959727</v>
+        <v>-0.2397991073280818</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1315000037781159</v>
+        <v>-0.1314863228981826</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.08626391425761008</v>
+        <v>-0.08626426318075293</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2509882709348245</v>
+        <v>0.2509799429119314</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.03020834176030108</v>
+        <v>-0.03021992381813353</v>
       </c>
       <c r="K5" t="n">
-        <v>0.09452510798107212</v>
+        <v>0.09451408112130161</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.197968595641625</v>
+        <v>-0.1979648915468615</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.05891463986612296</v>
+        <v>-0.05890202607779375</v>
       </c>
       <c r="N5" t="n">
-        <v>0.03103354591592346</v>
+        <v>0.03100547976321681</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.1907835607203862</v>
+        <v>-0.1907970361578747</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.1159299650229286</v>
+        <v>-0.1159018754676713</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.08363897507298565</v>
+        <v>-0.08362292288373305</v>
       </c>
     </row>
     <row r="6">
@@ -737,52 +742,52 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.09616081275407345</v>
+        <v>-0.09614653193185965</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.08689012223718132</v>
+        <v>-0.08689302559642334</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1024578075750018</v>
+        <v>-0.1024670641381996</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.2398266474959727</v>
+        <v>-0.2397991073280818</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.03721042529010902</v>
+        <v>-0.03718767038576265</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.05937870912899811</v>
+        <v>-0.05938452594167023</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.1448006009365439</v>
+        <v>-0.1448018569254628</v>
       </c>
       <c r="J6" t="n">
-        <v>0.008695295263876811</v>
+        <v>0.008683725739340505</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.2081574400351159</v>
+        <v>-0.2081644667275831</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.138922667529602</v>
+        <v>-0.1389216375642912</v>
       </c>
       <c r="M6" t="n">
-        <v>0.01997557948671905</v>
+        <v>0.0199954747388666</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.093335676495717</v>
+        <v>-0.09335273924387344</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.05617821370854102</v>
+        <v>-0.05618563871605308</v>
       </c>
       <c r="P6" t="n">
-        <v>-0.06376021901521188</v>
+        <v>-0.06371489933239169</v>
       </c>
       <c r="Q6" t="n">
-        <v>-0.01647267629549623</v>
+        <v>-0.01645366804369938</v>
       </c>
     </row>
     <row r="7">
@@ -792,52 +797,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.1096170365425155</v>
+        <v>-0.1096135312118162</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.02214946444162377</v>
+        <v>-0.02216192929112734</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.09036043017487924</v>
+        <v>-0.09035629639522169</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1315000037781159</v>
+        <v>-0.1314863228981826</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.03721042529010902</v>
+        <v>-0.03718767038576265</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.07321407010234855</v>
+        <v>-0.07321351346955851</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.1804060325878739</v>
+        <v>-0.180399089455289</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.1041084666123199</v>
+        <v>-0.1041034346500325</v>
       </c>
       <c r="K7" t="n">
-        <v>0.03648947028211201</v>
+        <v>0.0364932154418192</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.07872677260511023</v>
+        <v>-0.07874266436041658</v>
       </c>
       <c r="M7" t="n">
-        <v>0.04959708732323371</v>
+        <v>0.04960532270122138</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.09644337853568778</v>
+        <v>-0.09643832177911055</v>
       </c>
       <c r="O7" t="n">
-        <v>0.01033274161506323</v>
+        <v>0.01034127919725513</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.1265375402055921</v>
+        <v>-0.1265273947178983</v>
       </c>
       <c r="Q7" t="n">
-        <v>-0.1183413580160009</v>
+        <v>-0.1183325295838287</v>
       </c>
     </row>
     <row r="8">
@@ -847,52 +852,52 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.1444223790502424</v>
+        <v>-0.1444150351135369</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1667356404338387</v>
+        <v>0.1667294725423881</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.259347697756791</v>
+        <v>-0.2593522376531645</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.08626391425761008</v>
+        <v>-0.08626426318075293</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.05937870912899811</v>
+        <v>-0.05938452594167023</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.07321407010234855</v>
+        <v>-0.07321351346955851</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.01585277908054454</v>
+        <v>0.0158417657633572</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.07246100512590652</v>
+        <v>-0.07246574389619694</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.3187467420134847</v>
+        <v>-0.3187530391841286</v>
       </c>
       <c r="L8" t="n">
-        <v>0.123337949171726</v>
+        <v>0.1233329918496867</v>
       </c>
       <c r="M8" t="n">
-        <v>0.04739202893001999</v>
+        <v>0.04738778664711048</v>
       </c>
       <c r="N8" t="n">
-        <v>0.07912720969069084</v>
+        <v>0.07910756569897044</v>
       </c>
       <c r="O8" t="n">
-        <v>-0.08460103401759431</v>
+        <v>-0.08460971715277026</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.1170398364391229</v>
+        <v>-0.1170383085689743</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.1982911928096091</v>
+        <v>-0.1982865364427263</v>
       </c>
     </row>
     <row r="9">
@@ -902,52 +907,52 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.1096209680711279</v>
+        <v>-0.1096233308647602</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.1285428703752398</v>
+        <v>-0.1285498004740148</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.06117100019707069</v>
+        <v>-0.06118335721699146</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2509882709348245</v>
+        <v>0.2509799429119314</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.1448006009365439</v>
+        <v>-0.1448018569254628</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.1804060325878739</v>
+        <v>-0.180399089455289</v>
       </c>
       <c r="H9" t="n">
-        <v>0.01585277908054454</v>
+        <v>0.0158417657633572</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.03066222459164555</v>
+        <v>-0.03067438339290892</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.1972728637633153</v>
+        <v>-0.1972896533930862</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.2209132406089387</v>
+        <v>-0.220919288147655</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0132872134912887</v>
+        <v>0.01328029068344678</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2423363525825762</v>
+        <v>0.2423158155871055</v>
       </c>
       <c r="O9" t="n">
-        <v>-0.1191953422023948</v>
+        <v>-0.1192138946631024</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.01848415368200233</v>
+        <v>-0.01847965008483191</v>
       </c>
       <c r="Q9" t="n">
-        <v>-0.09305601182802407</v>
+        <v>-0.09305635670422695</v>
       </c>
     </row>
     <row r="10">
@@ -957,52 +962,52 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.04925957383564745</v>
+        <v>0.04925397476812462</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.04364093524481442</v>
+        <v>-0.04363539419800175</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1082913665113159</v>
+        <v>0.1082970332787706</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.03020834176030108</v>
+        <v>-0.03021992381813353</v>
       </c>
       <c r="F10" t="n">
-        <v>0.008695295263876811</v>
+        <v>0.008683725739340505</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.1041084666123199</v>
+        <v>-0.1041034346500325</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.07246100512590652</v>
+        <v>-0.07246574389619694</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.03066222459164555</v>
+        <v>-0.03067438339290892</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.1455028458792688</v>
+        <v>-0.1455025800917993</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1659014266280069</v>
+        <v>0.1659129006713242</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.1731900401056099</v>
+        <v>-0.1731987154598682</v>
       </c>
       <c r="N10" t="n">
-        <v>-0.1520017397161875</v>
+        <v>-0.152009884138331</v>
       </c>
       <c r="O10" t="n">
-        <v>0.006093886573959859</v>
+        <v>0.006090595189571032</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.1176788114641646</v>
+        <v>-0.1176836735582433</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.186512371200226</v>
+        <v>-0.1865129064845911</v>
       </c>
     </row>
     <row r="11">
@@ -1012,52 +1017,52 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.03502995936437731</v>
+        <v>0.03502673390221027</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.01414280009000239</v>
+        <v>-0.01414764888703375</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.05702846365874022</v>
+        <v>-0.05702766288127244</v>
       </c>
       <c r="E11" t="n">
-        <v>0.09452510798107212</v>
+        <v>0.09451408112130161</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.2081574400351159</v>
+        <v>-0.2081644667275831</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03648947028211201</v>
+        <v>0.0364932154418192</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.3187467420134847</v>
+        <v>-0.3187530391841286</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.1972728637633153</v>
+        <v>-0.1972896533930862</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.1455028458792688</v>
+        <v>-0.1455025800917993</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.04350823003569869</v>
+        <v>-0.04351163402090055</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.1908569086473705</v>
+        <v>-0.1908671862850687</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.01253419422843585</v>
+        <v>-0.0125450903479908</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.04021123267231936</v>
+        <v>-0.04021536648074502</v>
       </c>
       <c r="P11" t="n">
-        <v>0.04682604272749685</v>
+        <v>0.046820614345216</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.1091832983435418</v>
+        <v>0.1091803579959716</v>
       </c>
     </row>
     <row r="12">
@@ -1067,52 +1072,52 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.07146579894713018</v>
+        <v>-0.07146496179968009</v>
       </c>
       <c r="C12" t="n">
-        <v>0.08837535754800829</v>
+        <v>0.08833101272917128</v>
       </c>
       <c r="D12" t="n">
-        <v>0.07834398564172869</v>
+        <v>0.07834318818553589</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.197968595641625</v>
+        <v>-0.1979648915468615</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.138922667529602</v>
+        <v>-0.1389216375642912</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.07872677260511023</v>
+        <v>-0.07874266436041658</v>
       </c>
       <c r="H12" t="n">
-        <v>0.123337949171726</v>
+        <v>0.1233329918496867</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.2209132406089387</v>
+        <v>-0.220919288147655</v>
       </c>
       <c r="J12" t="n">
-        <v>0.1659014266280069</v>
+        <v>0.1659129006713242</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.04350823003569869</v>
+        <v>-0.04351163402090055</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.3913910774860525</v>
+        <v>-0.3914064279520365</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.02738765822092298</v>
+        <v>-0.02739195954151093</v>
       </c>
       <c r="O12" t="n">
-        <v>0.007460065363872877</v>
+        <v>0.007465197259808113</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.04120262766513379</v>
+        <v>-0.04120140813421686</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.1550298814911855</v>
+        <v>-0.155036141872387</v>
       </c>
     </row>
     <row r="13">
@@ -1122,52 +1127,52 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.1641235860623537</v>
+        <v>-0.1641089118636049</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.0003000413873512097</v>
+        <v>-0.0003130020767969113</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.138863151511475</v>
+        <v>-0.1388742670750134</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.05891463986612296</v>
+        <v>-0.05890202607779375</v>
       </c>
       <c r="F13" t="n">
-        <v>0.01997557948671905</v>
+        <v>0.0199954747388666</v>
       </c>
       <c r="G13" t="n">
-        <v>0.04959708732323371</v>
+        <v>0.04960532270122138</v>
       </c>
       <c r="H13" t="n">
-        <v>0.04739202893001999</v>
+        <v>0.04738778664711048</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0132872134912887</v>
+        <v>0.01328029068344678</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.1731900401056099</v>
+        <v>-0.1731987154598682</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.1908569086473705</v>
+        <v>-0.1908671862850687</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.3913910774860525</v>
+        <v>-0.3914064279520365</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1370518381360609</v>
+        <v>0.1370274396717936</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.2675499118726327</v>
+        <v>-0.2675608003310938</v>
       </c>
       <c r="P13" t="n">
-        <v>-0.09211247834669656</v>
+        <v>-0.09208574208925015</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.01762102006459238</v>
+        <v>0.01763185976389643</v>
       </c>
     </row>
     <row r="14">
@@ -1177,52 +1182,52 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.1415073162202437</v>
+        <v>-0.1415288649930178</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.01353837558253563</v>
+        <v>-0.01354378942813579</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1644678256392396</v>
+        <v>-0.1644710669846303</v>
       </c>
       <c r="E14" t="n">
-        <v>0.03103354591592346</v>
+        <v>0.03100547976321681</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.093335676495717</v>
+        <v>-0.09335273924387344</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.09644337853568778</v>
+        <v>-0.09643832177911055</v>
       </c>
       <c r="H14" t="n">
-        <v>0.07912720969069084</v>
+        <v>0.07910756569897044</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2423363525825762</v>
+        <v>0.2423158155871055</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.1520017397161875</v>
+        <v>-0.152009884138331</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.01253419422843585</v>
+        <v>-0.0125450903479908</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.02738765822092298</v>
+        <v>-0.02739195954151093</v>
       </c>
       <c r="M14" t="n">
-        <v>0.1370518381360609</v>
+        <v>0.1370274396717936</v>
       </c>
       <c r="N14" t="n">
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>-0.2063725365818479</v>
+        <v>-0.2063860167359353</v>
       </c>
       <c r="P14" t="n">
-        <v>-0.0594505348766715</v>
+        <v>-0.05946074594549591</v>
       </c>
       <c r="Q14" t="n">
-        <v>-0.1465362230453038</v>
+        <v>-0.1465537151430138</v>
       </c>
     </row>
     <row r="15">
@@ -1232,52 +1237,52 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.08680963195490667</v>
+        <v>0.08680258700840175</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.1815010411147558</v>
+        <v>-0.1815036698852637</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0207348601794416</v>
+        <v>0.02073547525390141</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1907835607203862</v>
+        <v>-0.1907970361578747</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.05617821370854102</v>
+        <v>-0.05618563871605308</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01033274161506323</v>
+        <v>0.01034127919725513</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.08460103401759431</v>
+        <v>-0.08460971715277026</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.1191953422023948</v>
+        <v>-0.1192138946631024</v>
       </c>
       <c r="J15" t="n">
-        <v>0.006093886573959859</v>
+        <v>0.006090595189571032</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.04021123267231936</v>
+        <v>-0.04021536648074502</v>
       </c>
       <c r="L15" t="n">
-        <v>0.007460065363872877</v>
+        <v>0.007465197259808113</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.2675499118726327</v>
+        <v>-0.2675608003310938</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.2063725365818479</v>
+        <v>-0.2063860167359353</v>
       </c>
       <c r="O15" t="n">
         <v>1</v>
       </c>
       <c r="P15" t="n">
-        <v>0.06714302103028884</v>
+        <v>0.06714034833759436</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1183165469587396</v>
+        <v>0.1183129237206472</v>
       </c>
     </row>
     <row r="16">
@@ -1287,52 +1292,52 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.09777156231626215</v>
+        <v>-0.09775477875327418</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.2443966077704177</v>
+        <v>-0.2443978567840111</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0128512565357735</v>
+        <v>-0.01285610416450294</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.1159299650229286</v>
+        <v>-0.1159018754676713</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.06376021901521188</v>
+        <v>-0.06371489933239169</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.1265375402055921</v>
+        <v>-0.1265273947178983</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.1170398364391229</v>
+        <v>-0.1170383085689743</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.01848415368200233</v>
+        <v>-0.01847965008483191</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.1176788114641646</v>
+        <v>-0.1176836735582433</v>
       </c>
       <c r="K16" t="n">
-        <v>0.04682604272749685</v>
+        <v>0.046820614345216</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.04120262766513379</v>
+        <v>-0.04120140813421686</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.09211247834669656</v>
+        <v>-0.09208574208925015</v>
       </c>
       <c r="N16" t="n">
-        <v>-0.0594505348766715</v>
+        <v>-0.05946074594549591</v>
       </c>
       <c r="O16" t="n">
-        <v>0.06714302103028884</v>
+        <v>0.06714034833759436</v>
       </c>
       <c r="P16" t="n">
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>-0.1216341524655653</v>
+        <v>-0.121608340118662</v>
       </c>
     </row>
     <row r="17">
@@ -1342,49 +1347,49 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.04353341731158855</v>
+        <v>0.04354939586290017</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.2406847034745391</v>
+        <v>-0.2406974875923396</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.134669307620711</v>
+        <v>-0.1346716575196713</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.08363897507298565</v>
+        <v>-0.08362292288373305</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.01647267629549623</v>
+        <v>-0.01645366804369938</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.1183413580160009</v>
+        <v>-0.1183325295838287</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.1982911928096091</v>
+        <v>-0.1982865364427263</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.09305601182802407</v>
+        <v>-0.09305635670422695</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.186512371200226</v>
+        <v>-0.1865129064845911</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1091832983435418</v>
+        <v>0.1091803579959716</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.1550298814911855</v>
+        <v>-0.155036141872387</v>
       </c>
       <c r="M17" t="n">
-        <v>0.01762102006459238</v>
+        <v>0.01763185976389643</v>
       </c>
       <c r="N17" t="n">
-        <v>-0.1465362230453038</v>
+        <v>-0.1465537151430138</v>
       </c>
       <c r="O17" t="n">
-        <v>0.1183165469587396</v>
+        <v>0.1183129237206472</v>
       </c>
       <c r="P17" t="n">
-        <v>-0.1216341524655653</v>
+        <v>-0.121608340118662</v>
       </c>
       <c r="Q17" t="n">
         <v>1</v>

</xml_diff>